<commit_message>
data: cierre dia 2026-07-21_1720 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/Planes AASS/sincargosjulio.xlsx
+++ b/01_INPUTS/Planes AASS/sincargosjulio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\Planes AASS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68EBF0FE-C2DD-4580-A8D2-202FAF9EDC76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9A058C-C8F4-4D35-8678-1F593FCEE011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{8398F70B-36A8-4A9F-A50B-4A31C9FEDDC3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{8398F70B-36A8-4A9F-A50B-4A31C9FEDDC3}"/>
   </bookViews>
   <sheets>
     <sheet name="plan frío" sheetId="1" r:id="rId1"/>
@@ -338,10 +338,10 @@
     <t>No cumple</t>
   </si>
   <si>
-    <t>Cjas Sin Cargos (El cazador)</t>
-  </si>
-  <si>
-    <t>Sin cargo vino el cazador en cualquier varietal</t>
+    <t>Cjas Sin Cargos (Los Arboles)</t>
+  </si>
+  <si>
+    <t>Sin cargo vino Los Arboles en cualquier varietal</t>
   </si>
 </sst>
 </file>
@@ -470,17 +470,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="33">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1472,94 +1462,94 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="33" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="32" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="31" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6">
-    <cfRule type="duplicateValues" dxfId="30" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7">
-    <cfRule type="duplicateValues" dxfId="29" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="duplicateValues" dxfId="28" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="duplicateValues" dxfId="27" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="26" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="25" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="24" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="duplicateValues" dxfId="23" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14">
-    <cfRule type="duplicateValues" dxfId="22" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="21" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="20" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="19" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="18" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="17" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="duplicateValues" dxfId="16" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="duplicateValues" dxfId="15" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="duplicateValues" dxfId="14" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23">
-    <cfRule type="duplicateValues" dxfId="13" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="12" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25">
-    <cfRule type="duplicateValues" dxfId="11" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26">
-    <cfRule type="duplicateValues" dxfId="10" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2217,7 +2207,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B32">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2344,10 +2334,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B5">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>